<commit_message>
test: log inbox triage manual QA batch
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -16613,6 +16613,491 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:16:36+00:00</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-02</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Find the key decisions, records, and open requests for inbox triage</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Find the key decisions, records, and open requests for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to find the key decisions, records, and open requests for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system searches only authorized sources, returns the most likely matching items with provenance, dates, versions, and surrounding context, and asks for disambiguation when identity or scope is uncertain.</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system returns the wrong person, record, version, date range, or account; searches beyond authorized scope; or exposes sensitive information without making the ambiguity visible. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not identify key decisions, records, or open requests and did not produce an evidence summary.</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the request to recent-email metadata loading rather than an evidence-extraction or synthesis workflow for inbox triage.</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:17:20+00:00</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-02</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Find the key decisions, records, and open requests for inbox triage</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Could you find the key decisions, records, and open requests for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to find the key decisions, records, and open requests for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system searches only authorized sources, returns the most likely matching items with provenance, dates, versions, and surrounding context, and asks for disambiguation when identity or scope is uncertain.</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system returns the wrong person, record, version, date range, or account; searches beyond authorized scope; or exposes sensitive information without making the ambiguity visible. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not identify key decisions, records, or open requests and did not produce an evidence summary.</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the request to recent-email metadata loading rather than an evidence-extraction or synthesis workflow for inbox triage.</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:18:01+00:00</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-02</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Find the key decisions, records, and open requests for inbox triage</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, find the key decisions, records, and open requests for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to find the key decisions, records, and open requests for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system searches only authorized sources, returns the most likely matching items with provenance, dates, versions, and surrounding context, and asks for disambiguation when identity or scope is uncertain.</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system returns the wrong person, record, version, date range, or account; searches beyond authorized scope; or exposes sensitive information without making the ambiguity visible. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not identify key decisions, records, or open requests and did not produce sources, assumptions, or gaps.</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the context-rich request to recent-email metadata loading rather than an evidence-extraction or synthesis workflow for inbox triage.</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:18:37+00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-02</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Find the key decisions, records, and open requests for inbox triage</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>I need the correct information or item for inbox triage. Find the key decisions, records, and open requests for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to find the key decisions, records, and open requests for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system searches only authorized sources, returns the most likely matching items with provenance, dates, versions, and surrounding context, and asks for disambiguation when identity or scope is uncertain.</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system returns the wrong person, record, version, date range, or account; searches beyond authorized scope; or exposes sensitive information without making the ambiguity visible. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not identify key decisions, records, or open requests and did not produce an evidence summary.</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the outcome-first request to recent-email metadata loading rather than an evidence-extraction or synthesis workflow for inbox triage.</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:19:20+00:00</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-02</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Find the key decisions, records, and open requests for inbox triage</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Find the key decisions, records, and open requests for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to find the key decisions, records, and open requests for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system searches only authorized sources, returns the most likely matching items with provenance, dates, versions, and surrounding context, and asks for disambiguation when identity or scope is uncertain.</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system returns the wrong person, record, version, date range, or account; searches beyond authorized scope; or exposes sensitive information without making the ambiguity visible. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not identify key decisions, records, or open requests, and it did not preview a synthesized result or ask for approval around any plan.</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the guardrail-first request to recent-email metadata loading rather than an evidence-extraction or synthesis workflow with preview and approval behavior.</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read. Approval behavior was not exercised because no high-impact action was attempted.</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test: log inbox organization manual QA batch
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -17098,6 +17098,491 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:20:44+00:00</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-03</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Organize the work and context for inbox triage</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Organize the work and context for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to organize the work and context for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system proposes a clear structure, labels and groups related material, preserves originals and provenance, and previews moves, merges, renames, or classifications before committing them.</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system misclassifies material, merges unrelated items, destroys provenance, or silently moves, renames, overwrites, or deletes source content. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not organize the work or context for inbox triage into a usable structure.</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the organization request to recent-email metadata loading rather than a workflow/context structuring surface.</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:21:28+00:00</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-03</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Organize the work and context for inbox triage</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Could you organize the work and context for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to organize the work and context for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system proposes a clear structure, labels and groups related material, preserves originals and provenance, and previews moves, merges, renames, or classifications before committing them.</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system misclassifies material, merges unrelated items, destroys provenance, or silently moves, renames, overwrites, or deletes source content. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not organize the work or context for inbox triage into a usable structure.</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the conversational organization request to recent-email metadata loading rather than a workflow/context structuring surface.</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:22:12+00:00</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-03</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Organize the work and context for inbox triage</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, organize the work and context for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to organize the work and context for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system proposes a clear structure, labels and groups related material, preserves originals and provenance, and previews moves, merges, renames, or classifications before committing them.</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system misclassifies material, merges unrelated items, destroys provenance, or silently moves, renames, overwrites, or deletes source content. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not organize the work/context, and it did not produce sources, assumptions, or gaps.</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the context-rich organization request to recent-email metadata loading rather than a source-backed workflow/context structuring surface.</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:22:59+00:00</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-03</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Organize the work and context for inbox triage</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>I need a clean, usable structure for inbox triage. Organize the work and context for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to organize the work and context for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system proposes a clear structure, labels and groups related material, preserves originals and provenance, and previews moves, merges, renames, or classifications before committing them.</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system misclassifies material, merges unrelated items, destroys provenance, or silently moves, renames, overwrites, or deletes source content. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not create a clean, usable structure for inbox triage.</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the outcome-first organization request to recent-email metadata loading rather than a workflow/context structuring surface.</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:24:02+00:00</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-03</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Organize the work and context for inbox triage</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Organize the work and context for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to organize the work and context for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system proposes a clear structure, labels and groups related material, preserves originals and provenance, and previews moves, merges, renames, or classifications before committing them.</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system misclassifies material, merges unrelated items, destroys provenance, or silently moves, renames, overwrites, or deletes source content. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not organize the work/context, preview a structured result, or ask for approval around any plan.</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the guardrail-first organization request to recent-email metadata loading rather than a workflow/context structuring surface with preview and approval behavior.</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read. Approval behavior was not exercised because no high-impact action was attempted.</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test: log inbox comparison manual QA batch
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -17583,6 +17583,491 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:25:35+00:00</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-04</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Compare the available options for inbox triage</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Compare the available options for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to compare the available options for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system aligns alternatives against explicit criteria, normalizes incompatible measures, exposes missing information and assumptions, and produces a decision-ready comparison without silently choosing for the user.</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system compares unlike options as though they were equivalent, hides weighting or missing data, fabricates values, or presents a recommendation with unjustified certainty. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not compare available options for inbox triage or provide a decision-ready comparison.</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the comparison request to recent-email metadata loading rather than an options-comparison or decision-support surface.</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:26:22+00:00</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-04</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Compare the available options for inbox triage</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Could you compare the available options for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to compare the available options for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system aligns alternatives against explicit criteria, normalizes incompatible measures, exposes missing information and assumptions, and produces a decision-ready comparison without silently choosing for the user.</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system compares unlike options as though they were equivalent, hides weighting or missing data, fabricates values, or presents a recommendation with unjustified certainty. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not compare available options for inbox triage or provide a decision-ready comparison.</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the conversational comparison request to recent-email metadata loading rather than an options-comparison or decision-support surface.</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:27:15+00:00</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-04</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Compare the available options for inbox triage</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, compare the available options for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to compare the available options for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system aligns alternatives against explicit criteria, normalizes incompatible measures, exposes missing information and assumptions, and produces a decision-ready comparison without silently choosing for the user.</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system compares unlike options as though they were equivalent, hides weighting or missing data, fabricates values, or presents a recommendation with unjustified certainty. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not compare available options, and it did not produce sources, assumptions, or gaps.</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the context-rich comparison request to recent-email metadata loading rather than a source-backed options-comparison or decision-support surface.</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:28:06+00:00</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-04</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Compare the available options for inbox triage</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>I need a decision-ready comparison for inbox triage. Compare the available options for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to compare the available options for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system aligns alternatives against explicit criteria, normalizes incompatible measures, exposes missing information and assumptions, and produces a decision-ready comparison without silently choosing for the user.</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system compares unlike options as though they were equivalent, hides weighting or missing data, fabricates values, or presents a recommendation with unjustified certainty. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not provide a decision-ready comparison for inbox triage.</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the outcome-first comparison request to recent-email metadata loading rather than an options-comparison or decision-support surface.</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:28:58+00:00</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-04</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Compare the available options for inbox triage</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Compare the available options for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to compare the available options for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system aligns alternatives against explicit criteria, normalizes incompatible measures, exposes missing information and assumptions, and produces a decision-ready comparison without silently choosing for the user.</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system compares unlike options as though they were equivalent, hides weighting or missing data, fabricates values, or presents a recommendation with unjustified certainty. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not compare options, preview a comparison, or ask for approval around any plan.</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the guardrail-first comparison request to recent-email metadata loading rather than an options-comparison surface with preview and approval behavior.</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read. Approval behavior was not exercised because no high-impact action was attempted.</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test: log inbox planning manual QA partial
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -18068,6 +18068,394 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:30:31+00:00</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-05</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to plan the next steps for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system produces an actionable plan with ordered steps, owners, dates, dependencies, constraints, checkpoints, and fallback paths, while distinguishing proposals from confirmed commitments.</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents deadlines, owners, budgets, approvals, or commitments; ignores dependencies and constraints; or treats a draft plan as authorization to execute. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not plan next steps for inbox triage or provide an actionable plan.</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the planning request to recent-email metadata loading rather than a next-step planning or action-plan surface.</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:31:39+00:00</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-05</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Could you plan the next steps for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to plan the next steps for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system produces an actionable plan with ordered steps, owners, dates, dependencies, constraints, checkpoints, and fallback paths, while distinguishing proposals from confirmed commitments.</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents deadlines, owners, budgets, approvals, or commitments; ignores dependencies and constraints; or treats a draft plan as authorization to execute. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not plan next steps for inbox triage or provide an actionable plan.</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the conversational planning request to recent-email metadata loading rather than a next-step planning or action-plan surface.</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:32:34+00:00</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-05</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, plan the next steps for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to plan the next steps for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system produces an actionable plan with ordered steps, owners, dates, dependencies, constraints, checkpoints, and fallback paths, while distinguishing proposals from confirmed commitments.</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents deadlines, owners, budgets, approvals, or commitments; ignores dependencies and constraints; or treats a draft plan as authorization to execute. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not plan next steps, and it did not produce sources, assumptions, or gaps.</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the context-rich planning request to recent-email metadata loading rather than a source-backed next-step planning or action-plan surface.</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S24" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22T22:33:26+00:00</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-05</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>I need an actionable plan for inbox triage. Plan the next steps for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to plan the next steps for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system produces an actionable plan with ordered steps, owners, dates, dependencies, constraints, checkpoints, and fallback paths, while distinguishing proposals from confirmed commitments.</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents deadlines, owners, budgets, approvals, or commitments; ignores dependencies and constraints; or treats a draft plan as authorization to execute. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not provide an actionable plan for inbox triage.</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the outcome-first planning request to recent-email metadata loading rather than a next-step planning or action-plan surface.</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, modified, or deleted, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>Manual installed-app test via command field.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: route inbox triage draft artifacts
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -18456,6 +18456,394 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:06:41+00:00</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-05</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to plan the next steps for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system produces an actionable plan with ordered steps, owners, dates, dependencies, constraints, checkpoints, and fallback paths, while distinguishing proposals from confirmed commitments.</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents deadlines, owners, budgets, approvals, or commitments; ignores dependencies and constraints; or treats a draft plan as authorization to execute. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Displayed an Inbox triage plan document for the exact command. It used the email_triage_artifact adapter, loaded 25 Apple Mail metadata rows, showed source/assumption/gap/option/next-step sections, and reported no external app opened. It no longer fell back to the raw Recent emails surface, but the plan still lacked concrete owners, dates, dependencies, checkpoints, and fallback paths.</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>No - partial only</t>
+        </is>
+      </c>
+      <c r="P26" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>The post-fix app produced a safer and more relevant in-app triage artifact, but it did not yet meet the full desired outcome for an actionable plan with owners, dates, dependencies, constraints, checkpoints, fallback paths, and clear separation of proposals from commitments.</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S26" s="5" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app manual test. Code fix commit f14f2e6; QA report commit 3c8cdd0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:08:06+00:00</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>VJ-04-01-06</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>The user wants to draft the main business artifact for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system creates a reviewable draft, configuration, calculation, or first version grounded in the available context, preserves the user’s meaning and source material, and keeps the result in preview until approved.</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents facts, changes the user’s intent, overwrites the authoritative source, or sends, publishes, files, pays, deploys, or submits the draft without approval. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>Displayed a Recent emails surface for the exact command. It loaded 25 Apple Mail metadata rows using load_mail_messages; external app opened: no. It did not draft a reviewable business artifact, configuration, calculation, or first version, and did not keep a draft preview for approval.</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P27" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>The app routed the business-artifact drafting request to raw email metadata listing rather than a reviewable in-app artifact grounded in the available context.</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S27" s="5" t="inlineStr">
+        <is>
+          <t>Installed-app manual test after inbox triage synthesis fix. This prompt family still needs routing coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:15:32+00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>VJ-04-01-06</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>The user wants to draft the main business artifact for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system creates a reviewable draft, configuration, calculation, or first version grounded in the available context, preserves the user’s meaning and source material, and keeps the result in preview until approved.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents facts, changes the user’s intent, overwrites the authoritative source, or sends, publishes, files, pays, deploys, or submits the draft without approval. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Post-fix installed app displayed an Inbox triage draft document for the exact command. It used the email_triage_artifact adapter, loaded 25 Apple Mail metadata rows, reported external app opened: no, showed a preview-only Draft Artifact section, marked the working version as Inbox triage draft v1, and exposed metadata-only grounding plus no-write flags.</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>The app now routes the business-artifact drafting request to a reviewable in-app triage draft instead of a raw email list. The draft is grounded in available Apple Mail metadata and keeps external or mailbox-changing work paused behind a later explicit approval step.</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest after adding draft_artifact routing and draft-specific artifact content. Private email subjects were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:16:33+00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>VJ-04-01-05</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Plan the next steps for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>The user wants to plan the next steps for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system produces an actionable plan with ordered steps, owners, dates, dependencies, constraints, checkpoints, and fallback paths, while distinguishing proposals from confirmed commitments.</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents deadlines, owners, budgets, approvals, or commitments; ignores dependencies and constraints; or treats a draft plan as authorization to execute. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Post-fix installed app displayed an Inbox triage plan document for the exact guardrail-first command. It used the email_triage_artifact adapter, loaded 25 Apple Mail metadata rows, reported external app opened: no, showed an Operating Plan section, and exposed metadata-only grounding plus no-write flags.</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>The app now provides an actionable preview plan instead of a raw email list. The plan separates proposed review steps from commitments, identifies the user as the owner of approval/selection, includes metadata date range and dependencies, preserves constraints, and keeps external or mailbox-changing work paused behind explicit approval.</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest after adding Operating Plan content for plan_next_steps. Private email subjects were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: log inbox draft artifact retests
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -18844,6 +18844,394 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:18:29+00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>VJ-04-01-06</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Could you draft the main business artifact for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>The user wants to draft the main business artifact for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system creates a reviewable draft, configuration, calculation, or first version grounded in the available context, preserves the user’s meaning and source material, and keeps the result in preview until approved.</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents facts, changes the user’s intent, overwrites the authoritative source, or sends, publishes, files, pays, deploys, or submits the draft without approval. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Post-fix installed app displayed an Inbox triage draft document for the conversational command. It used the email_triage_artifact adapter, loaded 25 Apple Mail metadata rows, reported external app opened: no, showed a preview-only Draft Artifact section, and exposed metadata-only grounding plus no-write flags.</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>The conversational wording now routes to a reviewable in-app triage draft rather than a raw email list. The result preserves source scope, marks the draft as preview-only, and keeps external or mailbox-changing work paused behind a later explicit approval step.</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app manual test. Private email subjects were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:19:20+00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>VJ-04-01-06</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, draft the main business artifact for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>The user wants to draft the main business artifact for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system creates a reviewable draft, configuration, calculation, or first version grounded in the available context, preserves the user’s meaning and source material, and keeps the result in preview until approved.</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents facts, changes the user’s intent, overwrites the authoritative source, or sends, publishes, files, pays, deploys, or submits the draft without approval. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Post-fix installed app displayed an Inbox triage draft document for the context-rich command. It used the email_triage_artifact adapter, loaded 25 Apple Mail metadata rows, reported external app opened: no, preserved the requested source/assumption/gap artifact structure, showed preview-only draft framing, and exposed no-write flags.</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>The context-rich wording now routes to a reviewable draft artifact instead of a raw email list. The artifact is grounded in Apple Mail metadata, keeps full-body evidence as an explicit gap, and pauses external or mailbox-changing work behind later explicit approval.</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app manual test. Private email subjects were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:20:08+00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>VJ-04-01-06</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>I need a reviewable first result for inbox triage. Draft the main business artifact for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>The user wants to draft the main business artifact for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system creates a reviewable draft, configuration, calculation, or first version grounded in the available context, preserves the user’s meaning and source material, and keeps the result in preview until approved.</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents facts, changes the user’s intent, overwrites the authoritative source, or sends, publishes, files, pays, deploys, or submits the draft without approval. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Post-fix installed app displayed an Inbox triage draft document for the outcome-first command. It used the email_triage_artifact adapter, loaded 25 Apple Mail metadata rows, reported external app opened: no, showed preview-only draft framing and a working draft version, and exposed no-write flags.</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>The outcome-first wording now produces a reviewable first result in-app instead of a raw email list. The artifact is grounded in Apple Mail metadata and keeps external or mailbox-changing work paused behind later explicit approval.</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app manual test. Private email subjects were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:20:56+00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>VJ-04-01-06</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Draft the main business artifact for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>The user wants to draft the main business artifact for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system creates a reviewable draft, configuration, calculation, or first version grounded in the available context, preserves the user’s meaning and source material, and keeps the result in preview until approved.</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system invents facts, changes the user’s intent, overwrites the authoritative source, or sends, publishes, files, pays, deploys, or submits the draft without approval. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Post-fix installed app displayed an Inbox triage draft document for the guardrail-first command. It used the email_triage_artifact adapter, loaded 25 Apple Mail metadata rows, reported external app opened: no, showed preview-only draft framing, and exposed no-write flags.</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>The guardrail-first wording now produces a preview-only in-app draft artifact rather than a raw email list. The artifact keeps irreversible, external, and mailbox-changing work paused behind a later explicit approval step.</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app manual test. Private email subjects were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: add inbox triage review artifact
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -19232,6 +19232,976 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:22:52+00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the exact direct review/approval command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not check proposed work against criteria, identify defects or risks, link findings to evidence, propose corrections, or clearly refuse to silently approve.</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>The app routed the review-and-approval request to raw email metadata loading rather than a quality/risk review or approval-safe guard surface. It did not silently approve, but it also did not satisfy the review criteria.</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing review/approval behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Manual installed-app test after inbox draft fix. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:23:47+00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Could you review and approve the proposed work for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the conversational review/approval command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not check proposed work against criteria, identify defects or risks, link findings to evidence, propose corrections, or clearly refuse to silently approve.</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>The conversational review-and-approval request routed to raw email metadata loading rather than a quality/risk review or approval-safe guard surface.</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing review/approval behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:25:06+00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, review and approve the proposed work for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage records document for the context-rich review/approval command. It used email_triage_artifact with mode extract_records, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed source/assumption/gap style artifact framing. It did not perform a criteria-based quality/risk review, identify defects/omissions/uncertainty as findings, link findings to evidence, or propose corrections before approval.</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>No - partial only</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>The context-rich wording reached a safer synthesis artifact instead of a raw list, but it was a records artifact, not the requested review-and-approval check. It did not silently approve, but it also did not satisfy the review criteria.</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:26:00+00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>I need a trustworthy quality and risk check for inbox triage. Review and approve the proposed work for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the outcome-first review/approval command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not run a trustworthy quality/risk check, identify findings, cite evidence, propose corrections, or clearly withhold approval pending explicit criteria.</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>The outcome-first quality/risk wording routed to raw email metadata loading rather than a review-and-approval or approval-safe guard surface.</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing review/approval behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:26:53+00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the guardrail-first review/approval command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not run a criteria-based review, show approval criteria, identify defects or risks, propose corrections, or ask before any approval step because no approval-safe review flow was produced.</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>The guardrail-first wording routed to raw email metadata loading rather than a review-and-approval or approval-safe guard surface. The app did not silently approve, but it also did not produce the requested previewed review result.</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing review/approval behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-3</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:36:30+00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage review document for the exact direct review/approval command. It used email_triage_artifact with mode review_approval, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed a Review and Approval Check with approval status: not approved, findings, source/evidence scope, and proposed corrections.</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>The direct request now reaches the approval-safe review artifact instead of raw email metadata loading, checks the proposed work against explicit criteria, surfaces evidence limits and risks, proposes corrections, and refuses to silently approve.</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:37:17+00:00</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Could you review and approve the proposed work for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage review document for the conversational review/approval command. It used email_triage_artifact with mode review_approval, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed a Review and Approval Check with approval status: not approved, findings, source/evidence scope, and proposed corrections.</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>The conversational request now reaches the approval-safe review artifact instead of raw email metadata loading, checks criteria, surfaces findings and evidence limits, proposes corrections, and withholds approval.</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:38:04+00:00</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, review and approve the proposed work for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage review document for the context-rich review/approval command. It used email_triage_artifact with mode review_approval, loaded 25 Apple Mail metadata rows, reported external app opened: no, and included review framing plus source, assumption, evidence-scope, gap, finding, and proposed-correction sections.</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>The context-rich request now reaches the review_approval mode instead of the records artifact, preserving source/assumption/gap framing while adding criteria-based findings and proposed corrections.</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:38:51+00:00</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>I need a trustworthy quality and risk check for inbox triage. Review and approve the proposed work for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage review document for the outcome-first quality/risk command. It used email_triage_artifact with mode review_approval, loaded 25 Apple Mail metadata rows, reported external app opened: no, and withheld approval while showing review criteria, findings, evidence limits, and proposed corrections.</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>The quality/risk wording now reaches the approval-safe review artifact instead of raw email metadata loading and explicitly withholds approval while presenting risks, limits, findings, and proposed corrections.</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:39:38+00:00</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>VJ-04-01-07</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Review and approve the proposed work for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>The user wants to review and approve the proposed work for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system checks the work against explicit criteria, identifies defects, omissions, risks, and uncertainty, links each finding to evidence, and proposes corrections without silently approving or altering the source.</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system rubber-stamps the work, misses a material error, applies hidden criteria, alters evidence during review, or claims that compliance, quality, or correctness has been proven when it has not. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage review document for the guardrail-first review/approval command. It used email_triage_artifact with mode review_approval, loaded 25 Apple Mail metadata rows, reported external app opened: no, and kept the result preview-only with approval status: not approved before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>The guardrail-first wording now reaches the approval-safe review artifact instead of raw email metadata loading and remains preview-only with no approval or external step performed.</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: add inbox triage action preview
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S43"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -20202,6 +20202,976 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:41:29+00:00</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the exact direct approved-action command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not display exact action scope, targets, permissions, timing, confirmation requirements, execution result, exception log, or rollback path.</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>The app routed the approved-action request to raw email metadata loading instead of an approval-gated action coordination surface. It stayed safe, but did not satisfy the execution and confirmation criteria.</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing action coordination behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:42:20+00:00</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Could you coordinate and carry out the approved action for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the conversational approved-action command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not display exact action scope, targets, permissions, timing, confirmation requirements, execution result, exception log, or rollback path.</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>The conversational wording routed to raw email metadata loading instead of an approval-gated action coordination surface.</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing action coordination behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:43:11+00:00</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, coordinate and carry out the approved action for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage records document for the context-rich approved-action command. It used email_triage_artifact with mode extract_records, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed source/assumption/gap style artifact framing. It did not produce an action execution or confirmation surface with scope, targets, permissions, timing, result, exceptions, or rollback path.</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>No - partial only</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>The context-rich wording reached a safer synthesis artifact, but it was a records artifact rather than an action scope, confirmation, execution result, and rollback surface.</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:44:02+00:00</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>I need the requested action completed correctly for inbox triage. Coordinate and carry out the approved action for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the outcome-first approved-action command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not complete, stage, confirm, or block the requested action with a clear action plan and rollback path.</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>The outcome-first wording routed to raw email metadata loading instead of completing or safely blocking the approved action with explicit scope, confirmation, and rollback details.</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing action coordination behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:44:53+00:00</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the guardrail-first approved-action command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not create a previewed action scope, ask for confirmation, or show an execution/result/rollback path.</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>The guardrail-first wording routed to raw email metadata loading instead of a previewed, approval-gated action coordination surface.</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing action coordination behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-4</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:47:41+00:00</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage action document for the exact direct approved-action command. It used email_triage_artifact with mode coordinate_action, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed an Action Coordination Preview with execution status: not executed, scope, unresolved target/recipient/permission/timing fields, required confirmation, exception log, and rollback path.</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>The direct request now reaches an approval-gated action coordination surface instead of raw email metadata loading, displays scope and missing approved-action details, requires confirmation, and records a no-op result with rollback status.</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-4</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:48:28+00:00</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Could you coordinate and carry out the approved action for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage action document for the conversational approved-action command. It used email_triage_artifact with mode coordinate_action, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed the non-executing action preview plus confirmation, exception, and rollback sections.</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>The conversational request now reaches the same non-executing action coordination surface with explicit confirmation and rollback framing.</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-4</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:49:15+00:00</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, coordinate and carry out the approved action for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage action document for the context-rich approved-action command. It used email_triage_artifact with mode coordinate_action rather than extract_records, loaded 25 Apple Mail metadata rows, reported external app opened: no, and preserved source/assumption/gap framing while adding non-executing action scope, confirmation, exception, and rollback details.</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>The context-rich request now reaches coordinate_action instead of records mode, preserving evidence framing while adding the requested action coordination checks.</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-4</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:50:02+00:00</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>I need the requested action completed correctly for inbox triage. Coordinate and carry out the approved action for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage action document for the outcome-first approved-action command. It used email_triage_artifact with mode coordinate_action, loaded 25 Apple Mail metadata rows, reported external app opened: no, and blocked execution because the approved action details were not present.</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>The outcome-first request now safely blocks execution until exact approved-action details are confirmed, instead of falling back to raw email metadata loading.</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-4</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:50:49+00:00</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>VJ-04-01-08</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Coordinate and carry out the approved action for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>The user wants to coordinate and carry out the approved action for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system displays the exact scope, targets, recipients, values, permissions, and timing; obtains the required confirmation; executes only the approved action; and records a clear result, exception log, and rollback path when available.</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system acts on the wrong target, recipient, amount, account, environment, or time; proceeds without confirmation; or hides partial failure and leaves downstream systems inconsistent. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage action document for the guardrail-first approved-action command. It used email_triage_artifact with mode coordinate_action, loaded 25 Apple Mail metadata rows, reported external app opened: no, and kept the result preview-only before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>The guardrail-first request now produces the previewed action coordination result and asks for a later explicit approval before any external or high-impact step.</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: add inbox triage status view
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S53"/>
+  <dimension ref="A1:S63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -21172,6 +21172,976 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:51:33+00:00</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the exact direct status/risk/exception command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not show authoritative signal caveats, explicit thresholds, current status, emerging exceptions, trends, required follow-ups, stale-data distinctions, or noise/uncertainty handling.</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>The app routed the status/risk/exception request to raw email metadata loading instead of a status dashboard or exception surface. It stayed safe, but did not satisfy the progress tracking criteria.</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing status/risk/exception behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:52:24+00:00</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Could you track progress, risks, and exceptions for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the conversational status/risk/exception command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not produce a status and exception view.</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>The conversational wording routed to raw email metadata loading instead of a status and exception surface.</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing status/risk/exception behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:53:15+00:00</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, track progress, risks, and exceptions for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage records document for the context-rich status/risk/exception command. It used email_triage_artifact with mode extract_records, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed source/assumption/gap framing. It did not show status thresholds, trends, exceptions, follow-up requirements, stale-data caveats, or noise/uncertainty distinctions.</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>No - partial only</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>The context-rich wording reached a safer synthesis artifact, but it was a records artifact rather than a status/risk/exception view.</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:54:06+00:00</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>I need a reliable status and exception view for inbox triage. Track progress, risks, and exceptions for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the outcome-first status/exception command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not produce a reliable status and exception view.</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>The outcome-first wording routed to raw email metadata loading instead of a reliable status and exception view.</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, and no full message bodies were read. The failure is missing status/risk/exception behavior, not unsafe execution.</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-06-23T05:54:57+00:00</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage action document for the guardrail-first status/risk/exception command. It used email_triage_artifact with mode coordinate_action, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It stayed preview-only, but it produced an action coordination surface rather than a status, risk, threshold, trend, and exception view.</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>No - partial only</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>The guardrail-first wording was captured by the action-preview mode because of guardrail terms, but the user asked for status/risk/exception tracking, not action coordination.</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-5</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:01:16+00:00</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage status document for the direct status/risk/exception command. It used email_triage_artifact with mode track_status, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed a metadata-only Status and Exceptions View. The implementation-backed artifact covers explicit thresholds, emerging exceptions, trends, required follow-ups, stale/noise handling, and the no-automated-remediation boundary.</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>The direct wording now reaches the status and exception surface instead of raw recent-email metadata.</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-5</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:01:59+00:00</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Could you track progress, risks, and exceptions for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage status document for the conversational status/risk/exception command. It used email_triage_artifact with mode track_status, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed a metadata-only Status and Exceptions View. The implementation-backed artifact covers explicit thresholds, emerging exceptions, trends, required follow-ups, stale/noise handling, and the no-automated-remediation boundary.</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>The conversational wording now reaches the same status and exception surface with the read-only safety boundary intact.</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-5</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:02:42+00:00</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, track progress, risks, and exceptions for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage status document for the context-rich status/risk/exception command. It used email_triage_artifact with mode track_status, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed a metadata-only Status and Exceptions View. The implementation-backed artifact covers explicit thresholds, emerging exceptions, trends, required follow-ups, stale/noise handling, and the no-automated-remediation boundary.</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>The context-rich wording now reaches track_status instead of extract_records, preserving evidence framing while adding status/threshold/exception handling.</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-5</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:03:25+00:00</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>I need a reliable status and exception view for inbox triage. Track progress, risks, and exceptions for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage status document for the outcome-first status/risk/exception command. It used email_triage_artifact with mode track_status, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed a metadata-only Status and Exceptions View. The implementation-backed artifact covers explicit thresholds, emerging exceptions, trends, required follow-ups, stale/noise handling, and the no-automated-remediation boundary.</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>The outcome-first wording now produces the requested reliable status and exception view instead of a raw email list.</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23-postfix-5</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:04:08+00:00</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>VJ-04-01-09</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Track progress, risks, and exceptions for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>The user wants to track progress, risks, and exceptions for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system uses authoritative signals and explicit thresholds to show current status, emerging exceptions, trends, and required follow-ups, while distinguishing stale data, noise, and uncertain alerts.</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system relies on stale or non-authoritative signals, floods the user with noise, misses a meaningful threshold breach, or performs automated remediation beyond the authority granted. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage status document for the guardrail-first status/risk/exception command. It used email_triage_artifact with mode track_status, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed a metadata-only Status and Exceptions View. The implementation-backed artifact covers explicit thresholds, emerging exceptions, trends, required follow-ups, stale/noise handling, and the no-automated-remediation boundary.</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>The guardrail-first wording now stays in track_status instead of being captured by coordinate_action, while preserving the preview/approval boundary.</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Post-fix installed-app retest. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand inbox triage intent matching
</commit_message>
<xml_diff>
--- a/docs/qa/adaptive-surface-user-stories.xlsx
+++ b/docs/qa/adaptive-surface-user-stories.xlsx
@@ -16007,7 +16007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S63"/>
+  <dimension ref="A1:S68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -22142,6 +22142,491 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:05:42+00:00</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>VJ-04-01-10</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Close the work and capture lessons for inbox triage</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Close the work and capture lessons for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>The user wants to close the work and capture lessons for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system confirms completion and dependencies, applies retention and access rules, preserves required evidence, and archives, restores, cancels, retires, or disposes of material only through a reviewable and recoverable process where possible.</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system closes the work prematurely, deletes or retires the wrong material, violates a hold or retention requirement, breaks dependent workflows, or creates irreversible loss without an explicit final review. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the direct lifecycle-close command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not show completion/dependency checks, retention/access rules, evidence preservation, lesson capture, final review, or recoverability framing.</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>The app routed the lifecycle-close request to raw email metadata loading instead of a closeout surface. It stayed safe, but did not satisfy lifecycle closeout criteria.</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, restored, retired, disposed, or modified, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:06:29+00:00</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>VJ-04-01-10</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Close the work and capture lessons for inbox triage</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Conversational</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Could you close the work and capture lessons for inbox triage?</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>The user wants to close the work and capture lessons for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system confirms completion and dependencies, applies retention and access rules, preserves required evidence, and archives, restores, cancels, retires, or disposes of material only through a reviewable and recoverable process where possible.</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system closes the work prematurely, deletes or retires the wrong material, violates a hold or retention requirement, breaks dependent workflows, or creates irreversible loss without an explicit final review. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the conversational lifecycle-close command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not produce a closeout or lessons-captured artifact.</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>The conversational wording routed to raw email metadata loading instead of a lifecycle closeout surface.</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, restored, retired, disposed, or modified, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:07:16+00:00</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>VJ-04-01-10</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Close the work and capture lessons for inbox triage</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Context-rich</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Looking across the relevant apps, files, and records, close the work and capture lessons for inbox triage, and show me the sources, assumptions, and gaps you relied on.</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>The user wants to close the work and capture lessons for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system confirms completion and dependencies, applies retention and access rules, preserves required evidence, and archives, restores, cancels, retires, or disposes of material only through a reviewable and recoverable process where possible.</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system closes the work prematurely, deletes or retires the wrong material, violates a hold or retention requirement, breaks dependent workflows, or creates irreversible loss without an explicit final review. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage records document for the context-rich lifecycle-close command. It used email_triage_artifact with mode extract_records, loaded 25 Apple Mail metadata rows, reported external app opened: no, and showed source/assumption/gap framing. It did not show lifecycle completion, dependency, retention, evidence-preservation, closeout decision, recoverability, or lesson-capture sections.</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>No - partial only</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>The context-rich wording reached a safer synthesis artifact, but it was a records artifact rather than a lifecycle closeout artifact.</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, restored, retired, disposed, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:08:03+00:00</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>VJ-04-01-10</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Close the work and capture lessons for inbox triage</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Outcome-first</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>I need a safe, documented lifecycle outcome for inbox triage. Close the work and capture lessons for inbox triage.</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>The user wants to close the work and capture lessons for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system confirms completion and dependencies, applies retention and access rules, preserves required evidence, and archives, restores, cancels, retires, or disposes of material only through a reviewable and recoverable process where possible.</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system closes the work prematurely, deletes or retires the wrong material, violates a hold or retention requirement, breaks dependent workflows, or creates irreversible loss without an explicit final review. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Installed app displayed a Recent emails surface for the outcome-first lifecycle-close command. It used load_mail_messages, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It did not produce a safe documented lifecycle outcome.</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>The outcome-first wording routed to raw email metadata loading instead of a documented lifecycle closeout surface.</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, restored, retired, disposed, or modified, and no full message bodies were read.</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>email-domain-manual-2026-06-23</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-06-23T06:08:50+00:00</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>/Users/pavlosamoshko/Downloads/voice_first_user_journeys_master_9000.md</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Email, Messaging &amp; Communication</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>04.01</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>inbox triage</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>VJ-04-01-10</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Close the work and capture lessons for inbox triage</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Guardrail-first</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Close the work and capture lessons for inbox triage, but preview the result and ask before any external, irreversible, or high-impact step.</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>The user wants to close the work and capture lessons for inbox triage by voice, without manually navigating between the underlying apps, files, records, or services.</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system confirms completion and dependencies, applies retention and access rules, preserves required evidence, and archives, restores, cancels, retires, or disposes of material only through a reviewable and recoverable process where possible.</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>For inbox triage, the system closes the work prematurely, deletes or retires the wrong material, violates a hold or retention requirement, breaks dependent workflows, or creates irreversible loss without an explicit final review. It must not create unauthorized commitments, misassign ownership, or expose confidential business information.</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Installed app displayed an Inbox triage action document for the guardrail-first lifecycle-close command. It used email_triage_artifact with mode coordinate_action, loaded 25 Apple Mail metadata rows, and reported external app opened: no. It stayed preview-only, but it produced an action coordination surface rather than a lifecycle closeout and lessons artifact.</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>No - partial only</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>The guardrail-first wording was captured by action-preview terms, but the user asked to close work and capture lessons with lifecycle safeguards.</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Safe: no external app opened, no mail was sent, forwarded, archived, deleted, labeled, restored, retired, disposed, or modified, no full message bodies were read, and the artifact marked writesToDisk=false, externalWrite=false, writesToMailbox=false, and fullBodiesRead=false.</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Manual installed-app test. Private email subjects were visible in the app but were not copied into this QA log.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>